<commit_message>
Update weekly ITF junior report
</commit_message>
<xml_diff>
--- a/data/swedish_entries.xlsx
+++ b/data/swedish_entries.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,7 +481,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Acceptance URL</t>
+          <t>Tournament URL</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Player URL</t>
         </is>
       </c>
     </row>
@@ -515,7 +520,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H2" t="n">
         <v>21.74</v>
@@ -535,55 +540,65 @@
           <t>https://www.itftennis.com/en/tournament/j100-moenchengladbach/ger/2026/j-j100-ger-2026-004/acceptance-list/</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/grace-bernstein/800668844/swe/jt/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J100</t>
+          <t>J60</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Moenchengladbach</t>
+          <t>Hillegom</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Boys</t>
+          <t>Girls</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Viggo Kalleskog</t>
+          <t>Mimmie Buchler</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2895</v>
+        <v>693</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="H3" t="n">
-        <v>23.36</v>
+        <v>23.07</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.itftennis.com/en/tournament/j100-moenchengladbach/ger/2026/j-j100-ger-2026-004/acceptance-list/</t>
+          <t>https://www.itftennis.com/en/tournament/j60-hillegom/ned/2026/j-j60-ned-2026-002/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/mimmie-buchler/800711385/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -605,11 +620,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mimmie Buchler</t>
+          <t>Nicole Saidizand</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>693</v>
+        <v>775</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -617,10 +632,10 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H4" t="n">
-        <v>23.07</v>
+        <v>22.91</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -635,6 +650,11 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j60-hillegom/ned/2026/j-j60-ned-2026-002/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/nicole-saidizand/800694981/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -656,11 +676,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nicole Saidizand</t>
+          <t>Emina Honic</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>775</v>
+        <v>814</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -671,7 +691,7 @@
         <v>10</v>
       </c>
       <c r="H5" t="n">
-        <v>22.91</v>
+        <v>23.15</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -686,6 +706,11 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j60-hillegom/ned/2026/j-j60-ned-2026-002/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/emina-honic/800749245/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -702,27 +727,25 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Girls</t>
+          <t>Boys</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Emina Honic</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>814</v>
-      </c>
+          <t>Jonathan Gabriel Nilsson</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Alt</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="H6" t="n">
-        <v>23.15</v>
+        <v>25.26</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -737,6 +760,11 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j60-hillegom/ned/2026/j-j60-ned-2026-002/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/jonathan-gabriel-nilsson/800845860/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -748,17 +776,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hillegom</t>
+          <t>Ioannina</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Boys</t>
+          <t>Girls</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Jonathan Gabriel Nilsson</t>
+          <t>Alexandra Vantola</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -768,10 +796,10 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="H7" t="n">
-        <v>25.26</v>
+        <v>31.47</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -785,7 +813,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://www.itftennis.com/en/tournament/j60-hillegom/ned/2026/j-j60-ned-2026-002/acceptance-list/</t>
+          <t>https://www.itftennis.com/en/tournament/j60-ioannina/gre/2026/j-j60-gre-2026-006/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/alexandra-vantola/800747958/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -802,25 +835,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Girls</t>
+          <t>Boys</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Alexandra Vantola</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>Spyridon Sioutas</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4218</v>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Alt</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H8" t="n">
-        <v>31.47</v>
+        <v>25.14</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -835,6 +870,11 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j60-ioannina/gre/2026/j-j60-gre-2026-006/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/spyridon-sioutas/800654611/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -846,58 +886,63 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ioannina</t>
+          <t>Nairobi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Boys</t>
+          <t>Girls</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Spyridon Sioutas</t>
+          <t>Lovisa Neselius</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4218</v>
+        <v>3201</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Alt</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="H9" t="n">
-        <v>25.14</v>
+        <v>30.77</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://www.itftennis.com/en/tournament/j60-ioannina/gre/2026/j-j60-gre-2026-006/acceptance-list/</t>
+          <t>https://www.itftennis.com/en/tournament/j60-nairobi/ken/2026/j-j60-ken-2026-003/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/lovisa-neselius/800643879/swe/jt/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J60</t>
+          <t>J30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nairobi</t>
+          <t>Banja Luka</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -907,22 +952,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Lovisa Neselius</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>3201</v>
-      </c>
+          <t>Emanuela Basic</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Alt</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H10" t="n">
-        <v>30.77</v>
+        <v>31.26</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -936,7 +979,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.itftennis.com/en/tournament/j60-nairobi/ken/2026/j-j60-ken-2026-003/acceptance-list/</t>
+          <t>https://www.itftennis.com/en/tournament/j30-banja-luka/bih/2026/j-j30-bih-2026-007/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/emanuela-basic/800809401/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -958,7 +1006,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Emanuela Basic</t>
+          <t>Neira Hadziomerovic</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -968,10 +1016,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H11" t="n">
-        <v>31.26</v>
+        <v>34.14</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -986,6 +1034,11 @@
       <c r="K11" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-banja-luka/bih/2026/j-j30-bih-2026-007/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/neira-hadziomerovic/800787369/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1002,25 +1055,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Girls</t>
+          <t>Boys</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Neira Hadziomerovic</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Viggo Salipurovic</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3903</v>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Alt</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="H12" t="n">
-        <v>34.14</v>
+        <v>23.92</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1035,6 +1090,11 @@
       <c r="K12" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-banja-luka/bih/2026/j-j30-bih-2026-007/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/viggo-salipurovic/800671572/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1056,22 +1116,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Viggo Salipurovic</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>3903</v>
-      </c>
+          <t>Valter Mandir</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>Alt</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="H13" t="n">
-        <v>23.92</v>
+        <v>25.64</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1086,6 +1144,11 @@
       <c r="K13" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-banja-luka/bih/2026/j-j30-bih-2026-007/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/valter-mandir/800709619/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1160,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Banja Luka</t>
+          <t>Izmir</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1107,20 +1170,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Valter Mandir</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Emil Curovic</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2376</v>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Alt</t>
+          <t>M</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H14" t="n">
-        <v>25.64</v>
+        <v>22.75</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1129,12 +1194,17 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.itftennis.com/en/tournament/j30-banja-luka/bih/2026/j-j30-bih-2026-007/acceptance-list/</t>
+          <t>https://www.itftennis.com/en/tournament/j30-izmir/tur/2026/j-j30-tur-2026-004/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/emil-curovic/800735502/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1216,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Izmir</t>
+          <t>Kaunas</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1156,11 +1226,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Emil Curovic</t>
+          <t>Patrick Eklund</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2376</v>
+        <v>1770</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1171,7 +1241,7 @@
         <v>12</v>
       </c>
       <c r="H15" t="n">
-        <v>22.75</v>
+        <v>22.23</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1180,12 +1250,17 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>https://www.itftennis.com/en/tournament/j30-izmir/tur/2026/j-j30-tur-2026-004/acceptance-list/</t>
+          <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/patrick-eklund/800692628/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1207,11 +1282,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Christian Gorgin</t>
+          <t>Oliver Wennerstad</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1272</v>
+        <v>2024</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1219,10 +1294,10 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H16" t="n">
-        <v>21.39</v>
+        <v>20.33</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1237,6 +1312,11 @@
       <c r="K16" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/oliver-wennerstad/800692529/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1258,22 +1338,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Patrick Eklund</t>
+          <t>Nils Preger</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1770</v>
+        <v>2626</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H17" t="n">
-        <v>22.23</v>
+        <v>22.03</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1288,6 +1368,11 @@
       <c r="K17" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/nils-preger/800668641/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1309,22 +1394,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Oliver Wennerstad</t>
+          <t>Noah Roberte</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2024</v>
+        <v>2820</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="H18" t="n">
-        <v>20.33</v>
+        <v>24.6</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1339,6 +1424,11 @@
       <c r="K18" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/noah-roberte/800728774/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1360,11 +1450,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nils Preger</t>
+          <t>Gustav Karlsson</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2626</v>
+        <v>2942</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1372,10 +1462,10 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H19" t="n">
-        <v>22.03</v>
+        <v>22.54</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1390,6 +1480,11 @@
       <c r="K19" t="inlineStr">
         <is>
           <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/gustav-karlsson/800738164/swe/jt/</t>
         </is>
       </c>
     </row>
@@ -1411,11 +1506,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Noah Roberte</t>
+          <t>Ludvig Ossian Sward</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2820</v>
+        <v>3374</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1423,10 +1518,10 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H20" t="n">
-        <v>24.6</v>
+        <v>21.62</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1443,155 +1538,9 @@
           <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>J30</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Kaunas</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Boys</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Gustav Karlsson</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>2942</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>8</v>
-      </c>
-      <c r="H21" t="n">
-        <v>22.54</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>J30</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Kaunas</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Boys</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Ludvig Ossian Sward</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>3374</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>14</v>
-      </c>
-      <c r="H22" t="n">
-        <v>21.62</v>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>2026-07-13</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>2026-07-18</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>https://www.itftennis.com/en/tournament/j30-kaunas/ltu/2026/j-j30-ltu-2026-004/acceptance-list/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>J30</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Szentes</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Boys</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Noel Hajduk</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Alt</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>13</v>
-      </c>
-      <c r="H23" t="n">
-        <v>26.75</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2026-07-19</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>https://www.itftennis.com/en/tournament/j30-szentes/hun/2026/j-j30-hun-2026-002/acceptance-list/</t>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.itftennis.com/en/players/ludvig-ossian-sward/800731644/swe/jt/</t>
         </is>
       </c>
     </row>

</xml_diff>